<commit_message>
Weekly tracked-horses update through 2026-09-13
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JnGbfoPwQdSmqcM2G92n96
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Adelaide River</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,36 +503,36 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46269</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Alphonsus Liguori</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46269</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,20 +558,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46269</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Comanche Brave</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,20 +597,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46269</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Equus Victor</t>
+          <t>Dancing Destiny</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -636,20 +636,20 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -659,36 +659,36 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Without Compromise</t>
+          <t>Folsom Blues</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -698,13 +698,13 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Green Empress</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,20 +714,20 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -737,13 +737,13 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46170</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Headmaster</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -753,20 +753,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,31 +776,31 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46184</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46170</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Leinster</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,20 +831,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -854,36 +854,36 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46170</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Monogram</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -893,13 +893,13 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46232</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -932,18 +932,18 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46170</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Headmaster</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -971,18 +971,18 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46266</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Port Ferdinand</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1010,13 +1010,13 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46232</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Sky Captain</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1049,13 +1049,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46232</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Snapretend</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1073,12 +1073,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1088,13 +1088,13 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46232</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Port Ferdinand</t>
+          <t>Star Of State</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1112,12 +1112,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1127,13 +1127,13 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46196</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Snellen</t>
+          <t>Summer Is Tomorrow</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1143,20 +1143,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gowran Park</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46284</v>
+        <v>46278</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1166,13 +1166,13 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46261</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Tennessee Stud</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1182,20 +1182,20 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46298</v>
+        <v>46278</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,36 +1205,36 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Thundering On</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1244,36 +1244,36 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="1" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Trustyourinstinct</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1283,13 +1283,13 @@
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="1" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Wemightakedlongway</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1299,20 +1299,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1322,13 +1322,13 @@
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="1" t="n">
-        <v>46238</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Imperial Merlin</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,15 +1338,15 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Sedgefield</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46312</v>
+        <v>46279</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1361,70 +1361,70 @@
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="1" t="n">
-        <v>46238</v>
+        <v>46273</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>The Institute</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>FINGER LAKES</t>
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>46312</v>
+        <v>46280</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>final entry</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>horsetracker</t>
+          <t>virtualstable</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="1" t="n">
-        <v>46238</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Divilabother</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Kelso</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>46312</v>
+        <v>46281</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1439,31 +1439,31 @@
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="1" t="n">
-        <v>46238</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Snellen</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Gowran Park</t>
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>46312</v>
+        <v>46284</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1478,6 +1478,318 @@
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="1" t="n">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-09-20
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LgL4Z9jScsLUNEdTd9aza6
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Adelaide River</t>
+          <t>Casamorati</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,15 +480,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Listowel</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -503,31 +503,31 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alphonsus Liguori</t>
+          <t>Eighteenth Smiles</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Joyous Heart</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,20 +558,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46170</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Comanche Brave</t>
+          <t>Magna Victoria</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,15 +597,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Listowel</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dancing Destiny</t>
+          <t>Mai Dahlia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -636,15 +636,15 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,13 +659,13 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Folsom Blues</t>
+          <t>Nail House</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,15 +675,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -698,13 +698,13 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Green Empress</t>
+          <t>Near Perfection</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,15 +714,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -737,36 +737,36 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Headmaster</t>
+          <t>Never The Same</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,36 +776,36 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Obscenity</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Listowel</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46232</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leinster</t>
+          <t>Rodeo Blues</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,15 +831,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Listowel</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -854,31 +854,31 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Monogram</t>
+          <t>Where Love Lives</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Fairyhouse</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -893,13 +893,13 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -909,15 +909,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Beverley</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46278</v>
+        <v>46287</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -932,13 +932,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46232</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Cristal Clere</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -948,15 +948,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Listowel</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46278</v>
+        <v>46287</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:32</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -971,31 +971,31 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46232</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Port Ferdinand</t>
+          <t>White Birch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Goodwood</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46278</v>
+        <v>46288</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1010,13 +1010,13 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46196</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sky Captain</t>
+          <t>Divilabother</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1026,20 +1026,20 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46278</v>
+        <v>46289</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1049,13 +1049,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Snapretend</t>
+          <t>Imperial Merlin</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Perth</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46278</v>
+        <v>46289</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1088,13 +1088,13 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Star Of State</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1104,20 +1104,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Haydock</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46278</v>
+        <v>46290</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>16:18</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1127,13 +1127,13 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Summer Is Tomorrow</t>
+          <t>Fortitudine</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1143,20 +1143,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Newmarket</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46278</v>
+        <v>46290</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1166,13 +1166,13 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tennessee Stud</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1182,20 +1182,20 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Newmarket</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46278</v>
+        <v>46298</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,36 +1205,36 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46276</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Thundering On</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46278</v>
+        <v>46312</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1244,36 +1244,36 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="1" t="n">
-        <v>46276</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Trustyourinstinct</t>
+          <t>Erdenali</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>46278</v>
+        <v>46312</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1283,13 +1283,13 @@
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="1" t="n">
-        <v>46276</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Wemightakedlongway</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1299,20 +1299,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>46278</v>
+        <v>46312</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1322,13 +1322,13 @@
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="1" t="n">
-        <v>46276</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Imperial Merlin</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,15 +1338,15 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sedgefield</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46279</v>
+        <v>46312</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1361,70 +1361,70 @@
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="1" t="n">
-        <v>46273</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>The Institute</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FINGER LAKES</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>46280</v>
+        <v>46312</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>final entry</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>virtualstable</t>
+          <t>horsetracker</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="1" t="n">
-        <v>46274</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Divilabother</t>
+          <t>White Birch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Kelso</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>46281</v>
+        <v>46312</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1439,31 +1439,31 @@
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="1" t="n">
-        <v>46275</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Snellen</t>
+          <t>Wimbledon Hawkeye</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Gowran Park</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>46284</v>
+        <v>46312</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1478,318 +1478,6 @@
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="1" t="n">
-        <v>46261</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Sparan Nua</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Newmarket</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>46298</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Benvenuto Cellini</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Erdenali</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>14:40</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Pierre Bonnard</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Puerto Rico</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>14:40</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Sparan Nua</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>14:05</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>White Birch</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Wimbledon Hawkeye</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-10-04
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YQWeMVdsgnxznYs3h7SV8X
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Count Palatine</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ayr</t>
+          <t>Longchamp</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46294</v>
+        <v>46299</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,13 +503,13 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46288</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Cristal Clere</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,20 +519,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Manaar</t>
+          <t>Dancing Saxon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,20 +558,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46287</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Divilabother</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,20 +597,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Uttoxeter</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,36 +620,36 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Greydreambeliever</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -659,36 +659,36 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Invincible Mind</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -698,36 +698,36 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Princess Child</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -737,13 +737,13 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -753,20 +753,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Longchamp</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,36 +776,36 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Spinning Around</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -815,36 +815,36 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46238</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Wo Wo Never</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46312</v>
+        <v>46299</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -854,6 +854,747 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cladach</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Estado De La Luna</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Forthethrillofit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gliondar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kaaranah</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Wolverhampton</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>declared</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Magnum Cor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Shaihaan</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Shay's Dream</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Killarney</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Without Compromise</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Southwell</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" s="1" t="n">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Kashala</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Thurles</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" s="1" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Manaar</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" s="1" t="n">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Snellen</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" s="1" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-10-11
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qwd4Zd61rdnukRtrF7Q15w
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Acula</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,36 +503,36 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cristal Clere</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dancing Saxon</t>
+          <t>Atomic City</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,15 +558,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -581,36 +581,36 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Divilabother</t>
+          <t>Beset</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uttoxeter</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Greydreambeliever</t>
+          <t>Chablis Rock</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -636,11 +636,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -659,31 +659,31 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Invincible Mind</t>
+          <t>Comfort Zone</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -698,13 +698,13 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Princess Child</t>
+          <t>Duchess Of Kenli</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,15 +714,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -737,13 +737,13 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Eighteenth Smiles</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -753,20 +753,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Longchamp</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,13 +776,13 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Spinning Around</t>
+          <t>Formous</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -792,15 +792,15 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wo Wo Never</t>
+          <t>Fratas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,15 +831,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46299</v>
+        <v>46306</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -854,13 +854,13 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cladach</t>
+          <t>Galileo Dame</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -870,15 +870,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -893,13 +893,13 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Estado De La Luna</t>
+          <t>Glyfada</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -909,15 +909,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -932,13 +932,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Forthethrillofit</t>
+          <t>Green Soul</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -948,15 +948,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -971,31 +971,31 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gliondar</t>
+          <t>Light Up The Dark</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1010,36 +1010,36 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kaaranah</t>
+          <t>Mawhibah</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wolverhampton</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1049,13 +1049,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Magnum Cor</t>
+          <t>Passenger</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1088,31 +1088,31 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shaihaan</t>
+          <t>Princess Child</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1127,31 +1127,31 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shay's Dream</t>
+          <t>Qualixia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Killarney</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1166,36 +1166,36 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Without Compromise</t>
+          <t>Seaxburh</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Southwell</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,36 +1205,36 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46295</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kashala</t>
+          <t>Seven Nation Army</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thurles</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1244,13 +1244,13 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="1" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Manaar</t>
+          <t>Shoda</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1260,20 +1260,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1283,13 +1283,13 @@
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="1" t="n">
-        <v>46287</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Snellen</t>
+          <t>Snapretend</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1299,20 +1299,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1322,13 +1322,13 @@
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>So Must I</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,20 +1338,20 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Naas</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46312</v>
+        <v>46306</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1361,31 +1361,31 @@
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="1" t="n">
-        <v>46238</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leicester</t>
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1400,70 +1400,70 @@
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="1" t="n">
-        <v>46238</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>The Institute</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>FINGER LAKES</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>final entry</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>horsetracker</t>
+          <t>virtualstable</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="1" t="n">
-        <v>46238</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>46312</v>
+        <v>46309</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1478,31 +1478,31 @@
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="1" t="n">
-        <v>46238</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Headmaster</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D28" s="1" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1517,31 +1517,31 @@
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" s="1" t="n">
-        <v>46238</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Kashala</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D29" s="1" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1556,18 +1556,18 @@
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" s="1" t="n">
-        <v>46238</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1595,6 +1595,240 @@
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>